<commit_message>
Refine feedback variable instructions and enhance TODO documentation
- Updated .env.example to clarify the creation of feedback variables for COPD, HF, Asthma, and Stroke topics, specifying that DEV variables are for local use.
- Revised INSTRUCTIONS.md to emphasize the distinction between DEV and LIVE feedback links, ensuring users understand where to set these variables.
- Modified new_topic.py to reflect changes in feedback variable instructions and streamline TODO.md generation for new topics.
- Adjusted TODO.md files for Asthma, COPD, HF, and Stroke to align with updated instructions for feedback workbook links.

These updates improve clarity and consistency in managing feedback variables across the Hub CPD application.
</commit_message>
<xml_diff>
--- a/copd/feedback/live.xlsx
+++ b/copd/feedback/live.xlsx
@@ -380,9 +380,158 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Useful</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Suggestion</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-31T15:52:45Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>copd S33US7</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Useful</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Really useful, thank you.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-31T15:54:42Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>copd S33US7</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Useful</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Thanks for a really useful presentation.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Heart failure</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-31T15:54:42Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>copd S33US7</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Useful</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Thanks, good reminder of the pitfalls of reliance on NEWS2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>